<commit_message>
build CRO audit agent phase one
</commit_message>
<xml_diff>
--- a/projects/cro-audit-agent/sites-to-audit.xlsx
+++ b/projects/cro-audit-agent/sites-to-audit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sites" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sites" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sites'!$A$1:$H$61</definedName>
@@ -563,11 +563,19 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>E:/Projects/devsplit-dev-os/projects/cro-audit-agent/output/cro-audit-results.xlsx</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="inlineStr"/>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
added gitignore and new tasks
</commit_message>
<xml_diff>
--- a/projects/cro-audit-agent/sites-to-audit.xlsx
+++ b/projects/cro-audit-agent/sites-to-audit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sites" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sites" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sites'!$A$1:$H$61</definedName>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="14"/>
     </font>
@@ -56,7 +62,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +79,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -113,13 +125,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -493,10 +508,10 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -561,7 +576,7 @@
           <t>furniture</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -573,110 +588,294 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>E:/Projects/devsplit-dev-os/projects/cro-audit-agent/output/cro-audit-results.xlsx</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr"/>
+          <t>output/working/lo-and-co-interiors</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>First run — completed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amazinggiantflowers.com</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Amazing Giant Flowers</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (home/event decor)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linneadesign.com/</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Linnea Design</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (home goods / stationery)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>http://boxwoodgift.com</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Boxwood Gift</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (gifting)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>http://melaninmeanings.com</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Melanin Meanings</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (confirm)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://smrutipens.com</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Smruti Pens</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (stationery / pens)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://aromaart.co/</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Aroma Art</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (home fragrance / candles)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nzitelli.com</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Nzitelli</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (confirm)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>http://www.outpatch.org</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Outpatch</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (confirm)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.placeofaroma.com</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Place of Aroma</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (home fragrance)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.packagemint.com</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Packagemint</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Set niche (packaging supplies)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -1180,102 +1379,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Sites to audit — input list for the CRO Audit Agent</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr"/>
+      <c r="A2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>The agent reads this file and audits each row where Status = Pending.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr"/>
+      <c r="A4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Columns</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t># — sequential number.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Store URL — the full homepage URL, including https://. Required.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Store Name — optional, for readability in reports.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Niche — one of: outfit/fashion, activewear, headwear, jewellery &amp; rings, handbags/purses/bags, cars &amp; auto, furniture, tents &amp; camping. Drives the niche-specific checks.</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Niche — one of: outfit/fashion, activewear, headwear, jewellery &amp; rings, handbags/purses/bags, cars &amp; auto, furniture, tents &amp; camping. Drives the niche-specific checks. Leave blank if none fit — only the universal checks then run.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Status — Pending / In progress / Done / Could not audit. The agent updates this.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Date Audited — filled by the agent when done.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Output File / Link — where the 92-row result for this store was written.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Notes — anything the team or agent wants to record.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr"/>
+      <c r="A14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>To add stores: paste one URL per row, set Niche, leave Status = Pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Screenshots are saved to output/working/&lt;store-slug&gt;/ (gitignored).</t>
         </is>
       </c>
     </row>

</xml_diff>